<commit_message>
feat: v0.4.0 世界海克斯·炼狱难度 (32 hexes, cap 8, protocol v12, infernal difficulty)
- 世界海克斯 24→32：新增永燃诅咒/死亡收割/和平契约/田野之怒/野性本能/中立统御/亡灵行军/恶魔契约 8 个高机制海克斯

- 全量数值上调（炼狱难度）：敌对/中立生物属性加强、通用诅咒加重、友好增益上调

- 每类装配上限 4→8（可配置，上限 32）；UI 分类区块双列网格

- 全玩家可见：存档级共享 + 全服广播，所有人即时看到他人抽取/取消

- 网络协议 VERSION=12（联机需全员同版本）

- 修复 .gitignore 误伤：补回 HexConfig.java / HexGameRules.java 源码跟踪

- 文档/内容总表/翻译同步 v0.4.0
</commit_message>
<xml_diff>
--- a/docs/海克斯工坊内容总表.xlsx
+++ b/docs/海克斯工坊内容总表.xlsx
@@ -10,7 +10,7 @@
     <sheet name="海克斯(124)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="装备(44)" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="锻造词条" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="世界海克斯(24)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="世界海克斯(32)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -73,7 +73,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -97,6 +97,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1404,27 +1407,27 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>hex_warden</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>守望者</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>棱彩</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>原版</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n">
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>原版</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="n">
         <v>5</v>
       </c>
       <c r="F26" s="2" t="inlineStr"/>
@@ -1440,27 +1443,27 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>hex_warmaster</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>战争领主</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" s="8" t="inlineStr">
         <is>
           <t>棱彩</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>原版</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="n">
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>原版</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="n">
         <v>5</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1480,27 +1483,27 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>hex_xp_overload</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>知识洪流</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>棱彩</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>原版</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n">
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>原版</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1516,27 +1519,27 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>hex_arena_sprint</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>疾风突进</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>白银</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>原版</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n">
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>原版</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="n">
         <v>8</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1552,27 +1555,27 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>hex_berserk</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>狂怒</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>白银</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
-        <is>
-          <t>原版</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n">
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>原版</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="n">
         <v>10</v>
       </c>
       <c r="F30" s="2" t="inlineStr"/>
@@ -1588,27 +1591,27 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>hex_crit_cascade</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>暴击瀑布</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="9" t="inlineStr">
         <is>
           <t>白银</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>原版</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n">
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>原版</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="n">
         <v>8</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1624,27 +1627,27 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>hex_dice_addict</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>掷骰狂人</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>白银</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
-        <is>
-          <t>原版</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="n">
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>原版</t>
+        </is>
+      </c>
+      <c r="E32" s="7" t="n">
         <v>8</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1660,27 +1663,27 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>hex_duelist</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>决斗者</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="9" t="inlineStr">
         <is>
           <t>白银</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
-        <is>
-          <t>原版</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="n">
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>原版</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="n">
         <v>8</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -8113,14 +8116,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="51" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8200,7 +8203,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>全体玩家获得的晶币 -10%</t>
+          <t>全体玩家获得的晶币 -20%</t>
         </is>
       </c>
     </row>
@@ -8227,7 +8230,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>全体玩家造成的伤害 -10%</t>
+          <t>全体玩家造成的伤害 -15%</t>
         </is>
       </c>
     </row>
@@ -8254,24 +8257,24 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>全体玩家最大生命 +4</t>
+          <t>全体玩家最大生命 +6</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>whx_ancient_weakness</t>
+          <t>whx_eternal_flame</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>远古衰弱</t>
+          <t>永燃诅咒</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>棱彩</t>
+          <t>黄金</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -8281,19 +8284,19 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>全体玩家最大生命 -6、造成伤害 -8%</t>
+          <t>全体玩家受到的伤害 +20%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>whx_genesis_pact</t>
+          <t>whx_ancient_weakness</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>创世契约</t>
+          <t>远古衰弱</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -8308,78 +8311,78 @@
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>全体玩家经验 +20%，世界海克斯抽取消耗经验减半</t>
+          <t>全体玩家最大生命 -10、造成伤害 -12%</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>whx_pasture_harmony</t>
+          <t>whx_death_harvest</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>牧场丰饶</t>
+          <t>死亡收割</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>白银</t>
+          <t>棱彩</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>友好</t>
+          <t>通用</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>友好生物移动速度 +10%</t>
+          <t>全体玩家造成的伤害 -15%，死亡时损失的经验翻倍</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>whx_herd_watchful</t>
+          <t>whx_genesis_pact</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>家畜警觉</t>
+          <t>创世契约</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>白银</t>
+          <t>棱彩</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>友好</t>
+          <t>通用</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>友好生物死亡时有 30% 概率不掉落战利品</t>
+          <t>全体玩家经验 +30%，世界海克斯抽取消耗经验 -60%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>whx_loyal_guard</t>
+          <t>whx_pasture_harmony</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>忠诚守护</t>
+          <t>牧场丰饶</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>黄金</t>
+          <t>白银</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -8389,24 +8392,24 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>友好生物攻击力 +2</t>
+          <t>友好生物移动速度 +10%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>whx_flock_shadow</t>
+          <t>whx_herd_watchful</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>牧群阴影</t>
+          <t>家畜警觉</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>黄金</t>
+          <t>白银</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -8416,24 +8419,24 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>友好生物最大生命 -4</t>
+          <t>友好生物死亡时有 50% 概率不掉落战利品</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>whx_beast_king</t>
+          <t>whx_loyal_guard</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>万兽之王</t>
+          <t>忠诚守护</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>棱彩</t>
+          <t>黄金</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -8443,24 +8446,24 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>友好生物最大生命 +8、攻击力 +2</t>
+          <t>友好生物攻击力 +2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>whx_angel_grace</t>
+          <t>whx_flock_shadow</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>天使眷顾</t>
+          <t>牧群阴影</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>棱彩</t>
+          <t>黄金</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -8470,132 +8473,132 @@
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>驯服生物每秒回复 0.5 点生命</t>
+          <t>友好生物最大生命 -6</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>whx_wild_spirit</t>
+          <t>whx_pacifist_oath</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
         <is>
-          <t>野性难驯</t>
+          <t>和平契约</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>白银</t>
+          <t>黄金</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>中立</t>
+          <t>友好</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>中立生物攻击力 +1</t>
+          <t>友好生物死亡时 100% 不掉落任何战利品</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>whx_vigilant_eye</t>
+          <t>whx_beast_king</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>警惕之眼</t>
+          <t>万兽之王</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>白银</t>
+          <t>棱彩</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>中立</t>
+          <t>友好</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>中立生物索敌范围 +30%</t>
+          <t>友好生物最大生命 +8、攻击力 +2</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>whx_pack_rage</t>
+          <t>whx_angel_grace</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>兽群狂暴</t>
+          <t>天使眷顾</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>黄金</t>
+          <t>棱彩</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>中立</t>
+          <t>友好</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>中立生物攻击力 +2</t>
+          <t>驯服生物每秒回复 1.0 点生命</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>whx_hunter_eye</t>
+          <t>whx_wrath_of_fields</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>猎人之眼</t>
+          <t>田野之怒</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>黄金</t>
+          <t>棱彩</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>中立</t>
+          <t>友好</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>玩家对中立生物造成的伤害 +15%</t>
+          <t>友好生物受到攻击时 100% 获得力量与速度反扑（5 秒）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>whx_apex_presence</t>
+          <t>whx_wild_spirit</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>终焉威压</t>
+          <t>野性难驯</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>棱彩</t>
+          <t>白银</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -8605,24 +8608,24 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>中立生物最大生命 +10、移速 +15%</t>
+          <t>中立生物攻击力 +2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>whx_peace_vision</t>
+          <t>whx_vigilant_eye</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>和平愿景</t>
+          <t>警惕之眼</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>棱彩</t>
+          <t>白银</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
@@ -8632,73 +8635,73 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>玩家对中立生物造成的伤害 +30%</t>
+          <t>中立生物索敌范围 +45%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>whx_shadow_power</t>
+          <t>whx_pack_rage</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>暗影强化</t>
+          <t>兽群狂暴</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>白银</t>
+          <t>黄金</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>敌对</t>
+          <t>中立</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>敌对生物最大生命 +2</t>
+          <t>中立生物攻击力 +3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>whx_fang_claw</t>
+          <t>whx_hunter_eye</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>尖牙利爪</t>
+          <t>猎人之眼</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>白银</t>
+          <t>黄金</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>敌对</t>
+          <t>中立</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>敌对生物攻击力 +1</t>
+          <t>玩家对中立生物造成的伤害 +20%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>whx_predator_swift</t>
+          <t>whx_wild_instinct</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>捕食者迅捷</t>
+          <t>野性本能</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
@@ -8708,51 +8711,51 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>敌对</t>
+          <t>中立</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>敌对生物移动速度 +20%</t>
+          <t>中立生物受到攻击时 50% 概率获得力量与速度反击（5 秒）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>whx_armor_shell</t>
+          <t>whx_apex_presence</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>装甲外壳</t>
+          <t>终焉威压</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>黄金</t>
+          <t>棱彩</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>敌对</t>
+          <t>中立</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>敌对生物护甲 +4</t>
+          <t>中立生物最大生命 +16、移速 +25%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>whx_abyss_awaken</t>
+          <t>whx_peace_vision</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>深渊觉醒</t>
+          <t>和平愿景</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
@@ -8762,39 +8765,255 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>敌对</t>
+          <t>中立</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>敌对生物最大生命 +12、攻击力 +4、移速 +15%</t>
+          <t>玩家对中立生物造成的伤害 +40%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
+          <t>whx_neutral_dominion</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>中立统御</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>棱彩</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>中立</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>中立生物最大生命 +6、攻击力 +4，玩家对中立生物造成的伤害 -30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>whx_shadow_power</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>暗影强化</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>白银</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>敌对生物最大生命 +4</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>whx_fang_claw</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>尖牙利爪</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>白银</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>敌对生物攻击力 +2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>whx_predator_swift</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>捕食者迅捷</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>黄金</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>敌对生物移动速度 +30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>whx_armor_shell</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>装甲外壳</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>黄金</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>敌对生物护甲 +6</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>whx_undead_march</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>亡灵行军</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>黄金</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>敌对生物死亡时 25% 概率在原地召唤 1 只同类</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>whx_abyss_awaken</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>深渊觉醒</t>
+        </is>
+      </c>
+      <c r="C31" s="9" t="inlineStr">
+        <is>
+          <t>棱彩</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="E31" s="7" t="inlineStr">
+        <is>
+          <t>敌对生物最大生命 +20、攻击力 +6、移速 +25%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
           <t>whx_blood_feast</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>血腥盛宴</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>棱彩</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>敌对</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
-        <is>
-          <t>敌对生物最大生命 +8；击杀敌对生物获得的晶币 +50%</t>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>敌对生物最大生命 +12；击杀敌对生物获得的晶币 +75%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>whx_demon_contract</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>恶魔契约</t>
+        </is>
+      </c>
+      <c r="C33" s="9" t="inlineStr">
+        <is>
+          <t>棱彩</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>敌对</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="inlineStr">
+        <is>
+          <t>敌对生物攻击吸血 30%，25% 概率对玩家施加虚弱与缓慢（5 秒）</t>
         </is>
       </c>
     </row>

</xml_diff>